<commit_message>
Cloud sign-in without a password: mail link, session from the link or from the URL hash, settings form
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Fgv6qWhgZF3MS8G3kaBei
</commit_message>
<xml_diff>
--- a/docs/bakasun-missing-info.xlsx
+++ b/docs/bakasun-missing-info.xlsx
@@ -864,17 +864,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>סיסמת ענן לוירג׳יני</t>
+          <t>ענן: כתובת האתר בפרויקט</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Supabase מוגדר. וירג׳יני צריכה סיסמה כדי שהנתונים יעלו לענן.</t>
+          <t>הכניסה לענן היא בקישור למייל, בלי סיסמה (נבנה 30/09). החשבון של info.virpro כבר קיים ומשויך לחברה. הקישור מהמייל כרגע מפנה ל-localhost:3000 כי כך מוגדר בפרויקט.</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>לקבוע סיסמה ולהעביר לה (לא לכתוב כאן)</t>
+          <t>פעם אחת, דקה: Supabase ← Authentication ← URL Configuration ← Site URL = https://roynaor-work.github.io/Bakasun/ (ולהוסיף אותה גם ל-Redirect URLs). עד אז יש מסלול חלופי: להדביק את הקישור בהגדרות.</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">

</xml_diff>